<commit_message>
Complete Accounts module test execution
</commit_message>
<xml_diff>
--- a/05-Bug-Reports/Accounts-Bug-Report-v1.0.xlsx
+++ b/05-Bug-Reports/Accounts-Bug-Report-v1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SIDDIQ\EspoCRM-QA-Automation\05-Bug-Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E10D4BE2-07D0-441A-85C9-2FAB6251A754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1474C6C8-9E4A-4BD8-A9E4-6D9199A2593D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
   <si>
     <t>Bug ID</t>
   </si>
@@ -33,25 +33,56 @@
     <t>Module</t>
   </si>
   <si>
-    <t>Description</t>
-  </si>
-  <si>
     <t>Severity</t>
   </si>
   <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
     <t>Accounts</t>
   </si>
   <si>
-    <t>No defects identified during Accounts module execution</t>
-  </si>
-  <si>
-    <t>Closed</t>
+    <t>BUG-ACC-001</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Steps to Reproduce</t>
+  </si>
+  <si>
+    <t>1.Open an existing Account.
+2.Modify the Description.
+3.Save the Account.
+4.Open Audit Log.
+5.Observe the recorded activities.
+6.Lock the Account.
+7.Unlock the Account.
+8.Open Audit Log again.</t>
+  </si>
+  <si>
+    <t>Expected Result</t>
+  </si>
+  <si>
+    <t>Actual Result</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>Account Unlock activity is not recorded in Audit Log</t>
+  </si>
+  <si>
+    <t>If Account Unlock is an auditable system activity, the Unlock action should be recorded in the Audit Log.</t>
+  </si>
+  <si>
+    <t>The Lock activity is recorded in the Audit Log, but the Unlock activity is not displayed.</t>
+  </si>
+  <si>
+    <t>Description field auditing is disabled, so the missing Description update is excluded from this defect. The Unlock activity requires further verification against EspoCRM's expected audit behavior.</t>
   </si>
 </sst>
 </file>
@@ -110,13 +141,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -398,48 +435,75 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="47.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.6640625" customWidth="1"/>
+    <col min="3" max="3" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="37.44140625" customWidth="1"/>
+    <col min="8" max="9" width="27.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>8</v>
+      <c r="E2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Accounts QA findings and ttraceability
</commit_message>
<xml_diff>
--- a/05-Bug-Reports/Accounts-Bug-Report-v1.0.xlsx
+++ b/05-Bug-Reports/Accounts-Bug-Report-v1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SIDDIQ\EspoCRM-QA-Automation\05-Bug-Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1474C6C8-9E4A-4BD8-A9E4-6D9199A2593D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AAB31EC-7C3F-44F4-BCB7-7799A5A22F25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>Bug ID</t>
   </si>
@@ -42,9 +42,6 @@
     <t>BUG-ACC-001</t>
   </si>
   <si>
-    <t>Title</t>
-  </si>
-  <si>
     <t>Medium</t>
   </si>
   <si>
@@ -54,16 +51,6 @@
     <t>Steps to Reproduce</t>
   </si>
   <si>
-    <t>1.Open an existing Account.
-2.Modify the Description.
-3.Save the Account.
-4.Open Audit Log.
-5.Observe the recorded activities.
-6.Lock the Account.
-7.Unlock the Account.
-8.Open Audit Log again.</t>
-  </si>
-  <si>
     <t>Expected Result</t>
   </si>
   <si>
@@ -73,23 +60,67 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>Account Unlock activity is not recorded in Audit Log</t>
-  </si>
-  <si>
-    <t>If Account Unlock is an auditable system activity, the Unlock action should be recorded in the Audit Log.</t>
-  </si>
-  <si>
-    <t>The Lock activity is recorded in the Audit Log, but the Unlock activity is not displayed.</t>
-  </si>
-  <si>
-    <t>Description field auditing is disabled, so the missing Description update is excluded from this defect. The Unlock activity requires further verification against EspoCRM's expected audit behavior.</t>
+    <t>Test Case / Source</t>
+  </si>
+  <si>
+    <t>Bug Title</t>
+  </si>
+  <si>
+    <t>Precondition</t>
+  </si>
+  <si>
+    <t>Environment</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Defect Classification</t>
+  </si>
+  <si>
+    <t>Post-execution exploratory investigation</t>
+  </si>
+  <si>
+    <t>Audit Log displays 'Locked' after Account is unlocked</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>An Account has been locked and is available to be unlocked.</t>
+  </si>
+  <si>
+    <t>The Audit Log should accurately record the unlock action as 'Unlocked'.</t>
+  </si>
+  <si>
+    <t>After the Account was unlocked, the Audit Log displayed 'Locked' for the action recorded after the unlock operation.</t>
+  </si>
+  <si>
+    <t>EspoCRM 10.0.4, Docker, Windows, local environment (http://localhost:8081)</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>Functional Defect</t>
+  </si>
+  <si>
+    <t>Confirmed during post-execution exploratory review. The existing execution summary had previously identified Unlock auditing as an investigation item.</t>
+  </si>
+  <si>
+    <t>1. Open an Account. 
+2. Lock the Account. 
+3. Open Audit Log and verify the lock entry. 
+4. Unlock the same Account.
+5. Open/refresh Audit Log. 
+6. Observe the entry generated for the unlock action.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -100,7 +131,14 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -141,19 +179,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -435,75 +467,111 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.6640625" customWidth="1"/>
-    <col min="3" max="3" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="28.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="37.44140625" customWidth="1"/>
-    <col min="8" max="9" width="27.109375" customWidth="1"/>
+    <col min="6" max="6" width="7.109375" customWidth="1"/>
+    <col min="7" max="7" width="37.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.109375" customWidth="1"/>
+    <col min="10" max="10" width="22" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="28.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>12</v>
-      </c>
     </row>
-    <row r="2" spans="1:9" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:14" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>9</v>
+      <c r="C2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>